<commit_message>
Fixing show done transaction check box toggle, Mark as done toggle, taxed and non taxed client lable.
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I206"/>
+  <dimension ref="A1:I296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3334,25 +3334,25 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>#1: كتيب A5 - 12 صفحة | Qty: 400 | Price: 9 | Total: 3600 | VAT: 540</t>
+          <t>#1: كتيب A5 - 12 صفحة | Qty: 250 | Price: 9 | Total: 2250 | VAT: 337.5; Discount: 0</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Quotation#197</t>
+          <t>Quotation#197, Invoice#381, QB#5170</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>3600</v>
+        <v>2250</v>
       </c>
       <c r="F95" t="n">
-        <v>540</v>
+        <v>337.5</v>
       </c>
       <c r="G95" t="n">
-        <v>4140</v>
+        <v>2587.5</v>
       </c>
       <c r="I95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>#1: استيكر دائري 5*5 سم - 01 | Qty: 250 | Price: 0.35 | Total: 87.5 | VAT: 0; #2: استيكر دائري 5*5 سم - 02 | Qty: 750 | Price: 0.35 | Total: 262.5 | VAT: 0; #3: استيكر دائري 5*5 سم - B | Qty: 200 | Price: 0.6 | Total: 120 | VAT: 0; #4: استيكر دائري 5*5 سم - M | Qty: 150 | Price: 0.62 | Total: 93 | VAT: 0; #5: استيكر دائري 5*5 سم - G | Qty: 100 | Price: 0.62 | Total: 62 | VAT: 0</t>
+          <t>#1: استيكر دائري 5*5 سم - 01 | Qty: 250 | Price: 0.35 | Total: 87.5 | VAT: 0; #2: استيكر دائري 5*5 سم - 02 | Qty: 750 | Price: 0.35 | Total: 262.5 | VAT: 0; #3: استيكر دائري 5*5 سم - B | Qty: 200 | Price: 0.6 | Total: 120 | VAT: 0; #4: استيكر دائري 5*5 سم - M | Qty: 150 | Price: 0.62 | Total: 93 | VAT: 0; #5: استيكر دائري 5*5 سم - G | Qty: 100 | Price: 0.62 | Total: 62 | VAT: 0; Discount: 0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3779,7 +3779,7 @@
         <v>625</v>
       </c>
       <c r="I108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -5185,7 +5185,6 @@
       <c r="G151" t="n">
         <v>414</v>
       </c>
-      <c r="H151" t="inlineStr"/>
       <c r="I151" t="b">
         <v>1</v>
       </c>
@@ -5203,12 +5202,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>#1: كتب لوبريف - 100 ورقة - تغليف فاخر | Qty: 52 | Price: 144 | Total: 7488 | VAT: 1123.2</t>
+          <t>#1: كتب لوبريف - 100 ورقة - تغليف فاخر | Qty: 52 | Price: 144 | Total: 7488 | VAT: 1123.2; Discount: 0</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Quotation#214, Invoice#374</t>
+          <t>Quotation#214, Invoice#374, QB#5172</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -5318,7 +5317,7 @@
         <v>550</v>
       </c>
       <c r="I155" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -6057,20 +6056,25 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>#1: استيكر مع شيت مغناطيس مقاس 40*25 سم | Qty: 4 | Price: 50 | Total: 200 | VAT: 30</t>
+          <t>#1: استيكر مع شيت مغناطيس مقاس 40*25 سم | Qty: 4 | Price: 57.5 | Total: 230 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>QB#5178</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="F178" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G178" t="n">
         <v>230</v>
       </c>
       <c r="I178" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179">
@@ -6115,7 +6119,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>#1: سند صرف - مقاس A4 - أصل فقط - طباعة ديجيتال | Qty: 500 | Price: .75 | Total: 375 | VAT: 56.25</t>
+          <t>#1: سند صرف - مقاس A4 - أصل فقط - طباعة ديجيتال | Qty: 500 | Price: .75 | Total: 375 | VAT: 56.25; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Invoice#382, QB#5195</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -6128,7 +6137,7 @@
         <v>431.25</v>
       </c>
       <c r="I180" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181">
@@ -6144,7 +6153,12 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>#1: استيكر العود الأزرق - شفاف - مقاس 3.5*4.5 سم | Qty: 240 | Price: 0.67 | Total: 160.8 | VAT: 0; #2: استيكر الشعار - شفاف - دائري - مقاس 6*6 سم | Qty: 240 | Price: .96 | Total: 230.39999999999998 | VAT: 0</t>
+          <t>#1: استيكر العود الأزرق - شفاف - مقاس 3.5*4.5 سم | Qty: 240 | Price: 0.671 | Total: 161.04 | VAT: 0; #2: استيكر الشعار - شفاف - دائري - مقاس 6*6 سم | Qty: 240 | Price: 0.959 | Total: 230.16 | VAT: 0; Discount: 1.2</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>QB#5174</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -6154,10 +6168,10 @@
         <v>0</v>
       </c>
       <c r="G181" t="n">
-        <v>391.2</v>
+        <v>390</v>
       </c>
       <c r="I181" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -6231,7 +6245,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>#1: لوحة أكريليك مقاس 37*27 سم - 6ملم مطبوع من الخلف | Qty: 1 | Price: 120 | Total: 120 | VAT: 18</t>
+          <t>#1: لوحة أكريليك مقاس 37*27 سم - 6ملم مطبوع من الخلف | Qty: 1 | Price: 120 | Total: 120 | VAT: 18; Discount: 0</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -6249,7 +6263,7 @@
         <v>138</v>
       </c>
       <c r="I184" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -6333,7 +6347,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>#1: لوحة أكريليك مفرغة مع بخاخ بوية لون أزرق | Qty: 1 | Price: 250 | Total: 250 | VAT: 0</t>
+          <t>#1: لوحة أكريليك مفرغة مع بخاخ بوية لون أزرق | Qty: 1 | Price: 250 | Total: 250 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>QB#5187</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -6346,7 +6365,7 @@
         <v>250</v>
       </c>
       <c r="I187" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -6527,20 +6546,25 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>#1: استيكر بلاستيك مقاس 70*100 سم - مركب على ورق مقوى | Qty: 1 | Price: 80 | Total: 80 | VAT: 0</t>
+          <t>#1: استيكر بلاستيك مقاس 70*100 سم - مركب على ورق مقوى | Qty: 1 | Price: 92 | Total: 92 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>QB#5180</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
       </c>
       <c r="G193" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="I193" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -6556,7 +6580,12 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>#1: رول اب مطبوع على بنر | Qty: 1 | Price: 150 | Total: 150 | VAT: 0</t>
+          <t>#1: رول اب مطبوع على بنر | Qty: 1 | Price: 150 | Total: 150 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>QB#5179</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -6569,7 +6598,7 @@
         <v>150</v>
       </c>
       <c r="I194" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -6585,20 +6614,25 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>#1: كروت ثيم اليوم الوطني مقاس 10*9 سم - نموذجين - ألف من كل نموذج | Qty: 2000 | Price: .20 | Total: 400 | VAT: 0</t>
+          <t>#1: كروت ثيم اليوم الوطني مقاس 10*9 سم - نموذجين - ألف من كل نموذج | Qty: 2000 | Price: 0.207 | Total: 414 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>QB#5177</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>400</v>
+        <v>414</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
       </c>
       <c r="G195" t="n">
-        <v>400</v>
+        <v>414</v>
       </c>
       <c r="I195" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -6701,14 +6735,19 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>#1: رول أب - طباعة على بنر | Qty: 1 | Price: 230 | Total: 230 | VAT: 0</t>
+          <t>#1: رول أب - طباعة على بنر | Qty: 1 | Price: 200 | Total: 200 | VAT: 30; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Invoice#388</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="F199" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G199" t="n">
         <v>230</v>
@@ -6759,20 +6798,25 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>#1: استيكر مقاس 15*10 سم - طباعة ديجيتال | Qty: 100 | Price: 1.04 | Total: 104 | VAT: 0; #2: استيكر مقاس 18*4 سم - طباعة ديجيتال | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #3: استيكر مقاس 13*7 سم - طباعة ديجيتال | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #4: استيكر مقاس 9*4 سم - طباعة ديجيتال | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #5: استيكر بلاستيك مقاس 5*5 سم | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #6: طباعة كرت مقاس 15*10 سم | Qty: 100 | Price: 1.15 | Total: 114.99999999999999 | VAT: 0</t>
+          <t>#1: استيكر مقاس 18*4 سم - طباعة ديجيتال | Qty: 100 | Price: 0.92 | Total: 92 | VAT: 0; #2: استيكر مقاس 18*4 سم - طباعة ديجيتال | Qty: 100 | Price: 0.92 | Total: 92 | VAT: 0; #3: استيكر مقاس 13*7 سم - طباعة ديجيتال | Qty: 100 | Price: 1.035 | Total: 103.5 | VAT: 0; #4: استيكر مقاس 9*4 سم - طباعة ديجيتال | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #5: استيكر بلاستيك مقاس 5*5 سم | Qty: 100 | Price: .92 | Total: 92 | VAT: 0; #6: طباعة كرت مقاس 15*10 سم | Qty: 100 | Price: 1.15 | Total: 115 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>QB#5184</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>587</v>
+        <v>586.5</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
       </c>
       <c r="G201" t="n">
-        <v>587</v>
+        <v>586.5</v>
       </c>
       <c r="I201" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -6807,7 +6851,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>دوت وان كافيه</t>
+          <t>قهوة دوت وان كافيه</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -6817,14 +6861,19 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>#1: رول أب على خامة بنر مقاس 85*200 سم | Qty: 3 | Price: 200 | Total: 600 | VAT: 90; Discount: 0</t>
+          <t>#1: رول أب على خامة بنر مقاس 85*200 سم | Qty: 3 | Price: 230 | Total: 690 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>QB#5181</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>600</v>
+        <v>690</v>
       </c>
       <c r="F203" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="G203" t="n">
         <v>690</v>
@@ -6918,6 +6967,2797 @@
       </c>
       <c r="I206" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>جمعية خياركم لتعليم القرآن والسنة والأخلاق السيئة</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>#1: بزنس كارد كوشيه وجهين | Qty: 200 | Price: 0.46 | Total: 92 | VAT: 0; #2: توصيل - محتمل | Qty: 1 | Price: 25 | Total: 25 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>117</v>
+      </c>
+      <c r="F207" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" t="n">
+        <v>117</v>
+      </c>
+      <c r="I207" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>شركة متحدة الاعمال التجارية</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>#1: ختم دائري R538 | Qty: 1 | Price: 100 | Total: 100 | VAT: 15; #2: ختم مستطيل S827 | Qty: 1 | Price: 100 | Total: 100 | VAT: 15; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Invoice#392</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>200</v>
+      </c>
+      <c r="F208" t="n">
+        <v>30</v>
+      </c>
+      <c r="G208" t="n">
+        <v>230</v>
+      </c>
+      <c r="I208" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>شركة أطياف البهجة</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>#1: لوحة أكريليك ذهبي - مفرغة  بالشعار- مقاس 120*100 سم | Qty: 1 | Price: 402.5 | Total: 402.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>QB#5207</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>402.5</v>
+      </c>
+      <c r="F209" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" t="n">
+        <v>402.5</v>
+      </c>
+      <c r="H209" t="inlineStr"/>
+      <c r="I209" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>مؤسسة رونق وفن التجارية</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>#1: ختم دائري معتمد - بالعنوان - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; #2: ختم دائري معتمد - فرع الطائف - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>276</v>
+      </c>
+      <c r="F210" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" t="n">
+        <v>276</v>
+      </c>
+      <c r="I210" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>فندق فيجين دايموند</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>#1: تفصيل ظرفبطاقة على ورق كرافت 300 جرام - طباعة لون واحد - وجهين | Qty: 5000 | Price: 0.59 | Total: 2950 | VAT: 442.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Quotation#222, Invoice#395, QB#5206</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>2950</v>
+      </c>
+      <c r="F211" t="n">
+        <v>442.5</v>
+      </c>
+      <c r="G211" t="n">
+        <v>3392.5</v>
+      </c>
+      <c r="I211" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>فرصة للأعمال والمشاريع - مصطفى مدارك</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2025-08-27</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>#1: ختم دائري R538 | Qty: 1 | Price: 120 | Total: 120 | VAT: 18; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>120</v>
+      </c>
+      <c r="F212" t="n">
+        <v>18</v>
+      </c>
+      <c r="G212" t="n">
+        <v>138</v>
+      </c>
+      <c r="I212" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>شركة العليمي اخوان</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>#1: استيكر مقاس 20*20 سم - مطبوع من الداخل | Qty: 5 | Price: 16 | Total: 80 | VAT: 12; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Invoice#396</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>80</v>
+      </c>
+      <c r="F213" t="n">
+        <v>12</v>
+      </c>
+      <c r="G213" t="n">
+        <v>92</v>
+      </c>
+      <c r="I213" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>بيت الاستشارات - وضاح طاهر</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>#1: كروت بزنس - كوشيه سلوفان مطفي وجهين | Qty: 200 | Price: 0.517 | Total: 103.4 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="F214" t="n">
+        <v>0</v>
+      </c>
+      <c r="G214" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="I214" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>علي عمر الدين</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>#1: ختم بورك فيك - S854 | Qty: 1 | Price: 70 | Total: 70 | VAT: 0; #2: انت متميزة - R538 | Qty: 1 | Price: 80 | Total: 80 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>150</v>
+      </c>
+      <c r="F215" t="n">
+        <v>0</v>
+      </c>
+      <c r="G215" t="n">
+        <v>150</v>
+      </c>
+      <c r="I215" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>لين - من طرف أنس الجيلاني</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>#1: كرت بزنس - كوشيه مطفي وجهين | Qty: 50 | Price: 1.38 | Total: 69 | VAT: 0; #2: كرت شكر - 15*10 سم | Qty: 50 | Price: 2.76 | Total: 138 | VAT: 0; #3: سليف علبة مقاس 10*80 سم | Qty: 30 | Price: 10 | Total: 300 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>507</v>
+      </c>
+      <c r="F216" t="n">
+        <v>0</v>
+      </c>
+      <c r="G216" t="n">
+        <v>507</v>
+      </c>
+      <c r="I216" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>دكتورة براء رجب</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>#1: استيكرات ديجيتال مقاس 10*4 سم | Qty: 100 | Price: 0.92 | Total: 92 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>92</v>
+      </c>
+      <c r="F217" t="n">
+        <v>0</v>
+      </c>
+      <c r="G217" t="n">
+        <v>92</v>
+      </c>
+      <c r="I217" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>مؤسسة أحمد حمزه الكيادي</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>#1: ختم مؤسسة دائري - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>138</v>
+      </c>
+      <c r="F218" t="n">
+        <v>0</v>
+      </c>
+      <c r="G218" t="n">
+        <v>138</v>
+      </c>
+      <c r="I218" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>قرطاسية المودة</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>#1: بنر شقة للإيجار مع 4 أخرام | Qty: 1 | Price: 30 | Total: 30 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>30</v>
+      </c>
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="G219" t="n">
+        <v>30</v>
+      </c>
+      <c r="I219" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>قرطاسية المودة</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>#1: استيكر ملف لجنة التميز | Qty: 1 | Price: 15 | Total: 15 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>15</v>
+      </c>
+      <c r="F220" t="n">
+        <v>0</v>
+      </c>
+      <c r="G220" t="n">
+        <v>15</v>
+      </c>
+      <c r="I220" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>أوقية - سلطان الغامدي</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2025-08-27</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>#1: طباعة وتركيب بنر - مقاس 1802*260 سم | Qty: 1 | Price: 2574 | Total: 2574 | VAT: 386.1; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Quotation#226</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>2574</v>
+      </c>
+      <c r="F221" t="n">
+        <v>386.1</v>
+      </c>
+      <c r="G221" t="n">
+        <v>2960.1</v>
+      </c>
+      <c r="I221" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>مجمع بيت الطب</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>#1: بطاقات ديجيتال | Qty: 2 | Price: 13.045 | Total: 26.09 | VAT: 3.91; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Invoice#405</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>26.09</v>
+      </c>
+      <c r="F222" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="G222" t="n">
+        <v>30</v>
+      </c>
+      <c r="I222" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>ريم الأحمدي - فلين</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>#1: فلين مواد صفية مقاس 50*70 سم | Qty: 3 | Price: 46 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>138</v>
+      </c>
+      <c r="F223" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" t="n">
+        <v>138</v>
+      </c>
+      <c r="I223" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>عيادة ابتسامة النجوم</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>#1: ختم الدكتورة شروق عابد - S852 | Qty: 1 | Price: 80 | Total: 80 | VAT: 0; #2: ختم الدكتورة شروق عابد - S854 | Qty: 1 | Price: 120 | Total: 120 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>200</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" t="n">
+        <v>200</v>
+      </c>
+      <c r="I224" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>مركز الطبي الدولي</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>#1: درع وسط - سندس الدباغ | Qty: 1 | Price: 280 | Total: 280 | VAT: 42; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Invoice#400</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>280</v>
+      </c>
+      <c r="F225" t="n">
+        <v>42</v>
+      </c>
+      <c r="G225" t="n">
+        <v>322</v>
+      </c>
+      <c r="I225" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>قريد ون - وفاء صالح</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>#1: استيكر Garde 1 - مقاس 9*4 سم - سيرادو | Qty: 20 | Price: 1.15 | Total: 23 | VAT: 0; #2: استيكر Garde 1 - مقاس 9*4 سم - جيهانغا | Qty: 20 | Price: 1.15 | Total: 23 | VAT: 0; #3: استيكر Garde 1 - مقاس 9*4 سم - بليند | Qty: 20 | Price: 1.15 | Total: 23 | VAT: 0; #4: استيكر Garde 1 - مقاس 9*4 سم - بليند اسبريسو | Qty: 20 | Price: 1.15 | Total: 23 | VAT: 0; #5: استيكر Garde 1 - مقاس 9*4 سم - هامبيلا | Qty: 20 | Price: 1.15 | Total: 23 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>115</v>
+      </c>
+      <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="n">
+        <v>115</v>
+      </c>
+      <c r="I226" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>مكتبة الهلال</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>#1: استيكر ملف | Qty: 2 | Price: 15 | Total: 30 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>30</v>
+      </c>
+      <c r="F227" t="n">
+        <v>0</v>
+      </c>
+      <c r="G227" t="n">
+        <v>30</v>
+      </c>
+      <c r="I227" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>مكتبة الهلال</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>#1: استيكر ملف | Qty: 1 | Price: 15 | Total: 15 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>15</v>
+      </c>
+      <c r="F228" t="n">
+        <v>0</v>
+      </c>
+      <c r="G228" t="n">
+        <v>15</v>
+      </c>
+      <c r="I228" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>مجمع نقاء الطبي</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>#1: بطاقات آي دي مع توصيل | Qty: 5 | Price: 46 | Total: 230 | VAT: 0; #2: توصيل | Qty: 1 | Price: 60 | Total: 60 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>290</v>
+      </c>
+      <c r="F229" t="n">
+        <v>0</v>
+      </c>
+      <c r="G229" t="n">
+        <v>290</v>
+      </c>
+      <c r="I229" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>شركة الوحدة للحديد</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>#1: ختم الشركة مستطيل - S827 | Qty: 1 | Price: 115 | Total: 115 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>115</v>
+      </c>
+      <c r="F230" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" t="n">
+        <v>115</v>
+      </c>
+      <c r="I230" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>آمنة أم محمد</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>#1: بنر مقاس 150*150 سم | Qty: 1 | Price: 150 | Total: 150 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>150</v>
+      </c>
+      <c r="F231" t="n">
+        <v>0</v>
+      </c>
+      <c r="G231" t="n">
+        <v>150</v>
+      </c>
+      <c r="I231" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>نجود - فلين</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>#1: فلين صغير مقاس 20*35 سم | Qty: 2 | Price: 23 | Total: 46 | VAT: 0; #2: فلين صغير مقاس 50*25 سم | Qty: 1 | Price: 34.5 | Total: 34.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0</v>
+      </c>
+      <c r="G232" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="I232" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>حلول التحلية</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>#1: توريد قلم فاخر مع طباعة يو في ملون بالشعار | Qty: 1000 | Price: 2.5 | Total: 2500 | VAT: 0; #2: توريد نوتبوك جلد مع طباعة يو في ملون بالشعار | Qty: 1000 | Price: 6.5 | Total: 6500 | VAT: 0; #3: توريد كيسقماش لون رمادي مع طباعة شعار لون واحد | Qty: 1000 | Price: 3.75 | Total: 3750 | VAT: 0; #4: تفصيل بروش بالشعار | Qty: 20 | Price: 20 | Total: 400 | VAT: 0; #5: تفصيل علم كبير مع سارية | Qty: 2 | Price: 650 | Total: 1300 | VAT: 0; #6: تفصيل علم صغير استاند للمكتب | Qty: 11 | Price: 150 | Total: 1650 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Quotation#220</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>16100</v>
+      </c>
+      <c r="F233" t="n">
+        <v>0</v>
+      </c>
+      <c r="G233" t="n">
+        <v>16100</v>
+      </c>
+      <c r="I233" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>حلول التحلية</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2025-08-07</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>#1: استيكرات Titan ASD 200 | Qty: 100 | Price: 1.85 | Total: 185 | VAT: 0; #2: استيكرات RAKA ST-441 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #3: استيكرات RAKA B-110 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #4: استيكرات RAKA B-111 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #5: استيكرات RAKA B-113 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #6: استيكرات RAKA C-220 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #7: استيكرات RAKA C-221 | Qty: 05 | Price: 1.85 | Total: 9.25 | VAT: 0; #8: استيكرات RAKA ST-440 | Qty: 50 | Price: 1.85 | Total: 92.5 | VAT: 0; #9: استيكرات Lavasol 5 | Qty: 10 | Price: 1.85 | Total: 18.5 | VAT: 0; #10: استيكرات Titan ASD 325 | Qty: 100 | Price: 1.85 | Total: 185 | VAT: 0; #11: استيكرات SpectraGuard 225 | Qty: 300 | Price: 1.85 | Total: 555 | VAT: 0; #12: استيكرات Titan ASD 200 | Qty: 500 | Price: 1.85 | Total: 925 | VAT: 0; #13: استيكرات SpectraGuard 300 | Qty: 100 | Price: 2.5 | Total: 250 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>2682.75</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
+        <v>2682.75</v>
+      </c>
+      <c r="I234" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>حلول التحلية</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2025-08-27</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>#1: كروت عبدالرحمن الأحمدي | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #2: كروت صفوت إبراهيم | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #3: كروت أيمن عصام | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #4: محمود حامد عبدالحميد | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>400</v>
+      </c>
+      <c r="F235" t="n">
+        <v>0</v>
+      </c>
+      <c r="G235" t="n">
+        <v>400</v>
+      </c>
+      <c r="I235" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>حلول التحلية</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2025-08-28</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>#1: كروت محمد العجمي | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #2: كروت مؤمن خطاب | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #3: كروت رشيد الغامدي | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; #4: كروت عزيز ياسين | Qty: 200 | Price: 0.5 | Total: 100 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>400</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" t="n">
+        <v>400</v>
+      </c>
+      <c r="I236" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>أم عبدالمحسن</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>#1: كروت مقاس A5 - طباعة وجه واحد | Qty: 50 | Price: 1 | Total: 50 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>QB#5188</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>50</v>
+      </c>
+      <c r="F237" t="n">
+        <v>0</v>
+      </c>
+      <c r="G237" t="n">
+        <v>50</v>
+      </c>
+      <c r="I237" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>مجموعة سدر</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>#1: استيكر مقاس 60*40 سم مع سلوفان مطفي | Qty: 3 | Price: 50 | Total: 150 | VAT: 22.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Invoice#402, QB#5190</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>150</v>
+      </c>
+      <c r="F238" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G238" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="I238" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>عبدالله جحرة - أنس الجيلاني</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>#1: ختم Passion &amp; Pleasure - S827 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>QB#5191</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>138</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0</v>
+      </c>
+      <c r="G239" t="n">
+        <v>138</v>
+      </c>
+      <c r="I239" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>حمد جمعان الغامدي</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2025-09-06</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>#1: ختم مشروع المدينة العمالية | Qty: 1 | Price: 140 | Total: 140 | VAT: 21; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Invoice#407, QB#5192</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>140</v>
+      </c>
+      <c r="F240" t="n">
+        <v>21</v>
+      </c>
+      <c r="G240" t="n">
+        <v>161</v>
+      </c>
+      <c r="I240" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>حمد جمعان الغامدي</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>#1: ختم المدينة الذكية R538 | Qty: 1 | Price: 120 | Total: 120 | VAT: 18; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Invoice#407, QB#5193</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>120</v>
+      </c>
+      <c r="F241" t="n">
+        <v>18</v>
+      </c>
+      <c r="G241" t="n">
+        <v>138</v>
+      </c>
+      <c r="I241" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>شركة كيان الماسية العقارية</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2025-09-03</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>#1: لوحة أكريليك مقاس 13.5*18 سم - مع شطف وتلميع جهتين - مع طباعة يو في | Qty: 1 | Price: 276 | Total: 276 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>276</v>
+      </c>
+      <c r="F242" t="n">
+        <v>0</v>
+      </c>
+      <c r="G242" t="n">
+        <v>276</v>
+      </c>
+      <c r="I242" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>عبدالرحمن الزهراني للذبائح الحرية</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>#1: استيكر ديجيتال مقاس 22*22 سم | Qty: 150 | Price: 1.6 | Total: 240 | VAT: 0; #2: استيكر ديجيتال مقاس 10*10 سم | Qty: 50 | Price: 0.4 | Total: 20 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>QB#5194</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>260</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" t="n">
+        <v>260</v>
+      </c>
+      <c r="I243" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>رانيا بن محفوظ</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>#1: كروت مقاس 3.5*5 سم - مع ترقيم من 1-200 - مع تخريم | Qty: 400 | Price: 0.5 | Total: 200 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>200</v>
+      </c>
+      <c r="F244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G244" t="n">
+        <v>200</v>
+      </c>
+      <c r="I244" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>شركة أراك</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2025-09-06</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>#1: بزنس كارد - مطفي وجهين | Qty: 1000 | Price: 0.16 | Total: 160 | VAT: 24; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Invoice#410</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>160</v>
+      </c>
+      <c r="F245" t="n">
+        <v>24</v>
+      </c>
+      <c r="G245" t="n">
+        <v>184</v>
+      </c>
+      <c r="I245" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>أمينة المطيري</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>#1: ختم بيضاوي O3555 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>138</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0</v>
+      </c>
+      <c r="G246" t="n">
+        <v>138</v>
+      </c>
+      <c r="I246" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>رانيا بن محفوظ</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2025-09-02</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>#1: كرت مقاس 10*15 سم - طباعة وجه واحد | Qty: 30 | Price: 3 | Total: 90 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>90</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" t="n">
+        <v>90</v>
+      </c>
+      <c r="I247" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>شوكلت ابتهال - EM Sweets</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2025-09-06</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>#1: استيكر ديجيتال - مقاس 6*9 سم | Qty: 300 | Price: 0.6 | Total: 180 | VAT: 0; #2: كروت ديجيتال - مقاس 6*9 سم - طباعة وجه واحد | Qty: 200 | Price: 0.6 | Total: 120 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>300</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" t="n">
+        <v>300</v>
+      </c>
+      <c r="I248" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>خبراء الفلاتر</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>#1: تغيير ختم مكسور بالجديد بدون طباعة | Qty: 1 | Price: 180 | Total: 180 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>180</v>
+      </c>
+      <c r="F249" t="n">
+        <v>0</v>
+      </c>
+      <c r="G249" t="n">
+        <v>180</v>
+      </c>
+      <c r="I249" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>مجمع بيت الطب</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>#1: طباعة بطاقة تعريفية (مشاعل خيبري + عبدالرحمن أحمد) | Qty: 2 | Price: 13.04 | Total: 26.08 | VAT: 3.91; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Invoice#406</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>26.08</v>
+      </c>
+      <c r="F250" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="G250" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I250" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>دكتورة هدى زاهر</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>#1: ختم جيب S722 | Qty: 1 | Price: 115 | Total: 115 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>115</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0</v>
+      </c>
+      <c r="G251" t="n">
+        <v>115</v>
+      </c>
+      <c r="I251" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>واحة التقنيات الحديثة</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>#1: ورق خطابات فاخر | Qty: 500 | Price: 0.8 | Total: 400 | VAT: 60; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Invoice#403</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>400</v>
+      </c>
+      <c r="F252" t="n">
+        <v>60</v>
+      </c>
+      <c r="G252" t="n">
+        <v>460</v>
+      </c>
+      <c r="I252" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>بدوري - محمد العمري</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>#1: فلين 70*100 سم | Qty: 1 | Price: 92 | Total: 92 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>92</v>
+      </c>
+      <c r="F253" t="n">
+        <v>0</v>
+      </c>
+      <c r="G253" t="n">
+        <v>92</v>
+      </c>
+      <c r="I253" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>نادي الاتحاد</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>#1: طباعة فابريك باك لايت مقاس 100*122 سم | Qty: 4 | Price: 160 | Total: 640 | VAT: 96; #2: طباعة فابريك باك لايت مقاس 97*222 سم | Qty: 4 | Price: 290 | Total: 1160 | VAT: 174; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Quotation#231</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F254" t="n">
+        <v>270</v>
+      </c>
+      <c r="G254" t="n">
+        <v>2070</v>
+      </c>
+      <c r="I254" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>كابلات بحرة</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>#1: ختم اسم Mamdouh AlHadeeya | Qty: 1 | Price: 50 | Total: 50 | VAT: 7.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Invoice#409, QB#5199</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>50</v>
+      </c>
+      <c r="F255" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G255" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="I255" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>شركة موفينترا</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>#1: ختم دائري R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; #2: ورق خطابات فاخر | Qty: 100 | Price: 1.725 | Total: 172.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="F256" t="n">
+        <v>0</v>
+      </c>
+      <c r="G256" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="I256" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>شاي فال</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>#1: استيكر منيو مقاس 34*75 سم | Qty: 1 | Price: 50 | Total: 50 | VAT: 7.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>50</v>
+      </c>
+      <c r="F257" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G257" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="I257" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>أم عبدالمحسن</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>#1: كتاب 97 صفحة - تغليف سلك - داخلي وودفري 100 جرام | Qty: 1 | Price: 80 | Total: 80 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>QB#5196</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>80</v>
+      </c>
+      <c r="F258" t="n">
+        <v>0</v>
+      </c>
+      <c r="G258" t="n">
+        <v>80</v>
+      </c>
+      <c r="I258" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>سعيد القرني</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>#1: ختم S827 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>138</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0</v>
+      </c>
+      <c r="G259" t="n">
+        <v>138</v>
+      </c>
+      <c r="I259" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>المنارة الذهبية</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2025-08-16</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>#1: بروشور إي ثري مطوي من النص مطبوع وجهين على 150 جرام | Qty: 500 | Price: 2 | Total: 1000 | VAT: 150; #2: تصاميم تعديل بروشور ودعوة نموذجين | Qty: 1 | Price: 250 | Total: 250 | VAT: 37.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>QB#5197</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F260" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="G260" t="n">
+        <v>1437.5</v>
+      </c>
+      <c r="I260" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>المنارة الذهبية</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2025-08-17</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>#1: بطاقات آي دي مع حبل وجيب | Qty: 6 | Price: 60 | Total: 360 | VAT: 54; #2: كرت وجهين مسلفن مطفي | Qty: 1000 | Price: 0.16 | Total: 160 | VAT: 24; #3: بوك طلبية عميل - أصل فقط - شد 100 - ترقيم 001 - طباعة لون واحد | Qty: 10 | Price: 20 | Total: 200 | VAT: 30; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>QB#5198</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>720</v>
+      </c>
+      <c r="F261" t="n">
+        <v>108</v>
+      </c>
+      <c r="G261" t="n">
+        <v>828</v>
+      </c>
+      <c r="I261" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>حلول التحلية</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>#1: RO Plant Site Visit بوك إي فور - أصل + صورتين - لون أزرق - ترقيم من 0001 | Qty: 10 | Price: 28 | Total: 280 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>280</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0</v>
+      </c>
+      <c r="G262" t="n">
+        <v>280</v>
+      </c>
+      <c r="I262" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>المحاور الأربعة</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>#1: كتاب حلزوني مقاس A3 - ورق داخلي 150 جرام - مشروع السيد سلطان سعيد - 87 صفحة | Qty: 1 | Price: 87 | Total: 87 | VAT: 13.05; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Invoice#408, QB#5205</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>87</v>
+      </c>
+      <c r="F263" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="G263" t="n">
+        <v>100.05</v>
+      </c>
+      <c r="I263" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>رماه</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>#1: بطاقات آي دي | Qty: 4 | Price: 80.5 | Total: 322 | VAT: 48.3; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>322</v>
+      </c>
+      <c r="F264" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="G264" t="n">
+        <v>370.3</v>
+      </c>
+      <c r="I264" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>روضة حنان الورد</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>#1: لوحة اكريليك مقاس 30*25 سم - سماكة 6 ملم - مع 4 أخرام ومسامير | Qty: 1 | Price: 115 | Total: 115 | VAT: 0; #2: توصيل | Qty: 1 | Price: 15 | Total: 15 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>130</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0</v>
+      </c>
+      <c r="G265" t="n">
+        <v>130</v>
+      </c>
+      <c r="I265" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>#1: طباعة مسلفن مطفي مع دايكت وكفراج - باسم فالح الروقي | Qty: 1000 | Price: 1.6 | Total: 1600 | VAT: 240; #2: طباعة مسلفن مطفي مع دايكت وكفراج - باسم العيادة | Qty: 1000 | Price: 1.6 | Total: 1600 | VAT: 240; #3: طباعة مسلفن مطفي مع دايكت وكفراج - باسم سلمى الشيخ | Qty: 1000 | Price: 1.6 | Total: 1600 | VAT: 240; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F266" t="n">
+        <v>720</v>
+      </c>
+      <c r="G266" t="n">
+        <v>5520</v>
+      </c>
+      <c r="I266" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2025-09-01</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>#1: طباعة أبواك (خدمات تجميل) مقاس 14.5*21 سم - طباعة لون واحد (بني) - أصل + صورة - ترقيم من 001 | Qty: 10 | Price: 20 | Total: 200 | VAT: 30; #2: طباعة أبواك (خدمات أسنان) مقاس 14.5*21 سم - طباعة لون واحد (بني) - أصل + صورة - ترقيم من 001 | Qty: 10 | Price: 20 | Total: 200 | VAT: 30; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>400</v>
+      </c>
+      <c r="F267" t="n">
+        <v>60</v>
+      </c>
+      <c r="G267" t="n">
+        <v>460</v>
+      </c>
+      <c r="I267" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>#1: تفصيل علم مكتبي صغير مع استاند | Qty: 6 | Price: 200 | Total: 1200 | VAT: 180; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F268" t="n">
+        <v>180</v>
+      </c>
+      <c r="G268" t="n">
+        <v>1380</v>
+      </c>
+      <c r="I268" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>#1: تفصيل استاند مكتبي مقاس 30*30 سم - مطبوع يو في مع طبقة أكريليك ذهبي بالإيطار والشعارات | Qty: 1 | Price: 250 | Total: 250 | VAT: 37.5; #2: كوبون مقاس 21*7 سم - مع شرشرة وترقيم - بوك شد 50 | Qty: 16 | Price: 18 | Total: 288 | VAT: 43.2; #3: بروشور خدمات مقاس A5 - وجهين | Qty: 500 | Price: 0.6 | Total: 300 | VAT: 45; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>838</v>
+      </c>
+      <c r="F269" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="G269" t="n">
+        <v>963.7</v>
+      </c>
+      <c r="I269" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>#1: بروشور خدمات مقاس A5 - وجهين | Qty: 1000 | Price: 0.6 | Total: 600 | VAT: 90; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>600</v>
+      </c>
+      <c r="F270" t="n">
+        <v>90</v>
+      </c>
+      <c r="G270" t="n">
+        <v>690</v>
+      </c>
+      <c r="I270" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>#1: بروشور خدمات إنجليزي مقاس A5 - وجهين | Qty: 200 | Price: 0.6 | Total: 120 | VAT: 18; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>120</v>
+      </c>
+      <c r="F271" t="n">
+        <v>18</v>
+      </c>
+      <c r="G271" t="n">
+        <v>138</v>
+      </c>
+      <c r="I271" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>مجمع قبل وبعد</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>#1: بروشور خدمات مقاس A5 - وجهين | Qty: 500 | Price: 0.6 | Total: 300 | VAT: 45; #2: كوبون مقاس 21*7 سم - مع شرشرة وترقيم - بوك شد 50 | Qty: 6 | Price: 18 | Total: 108 | VAT: 16.2; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Quotation#234</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>408</v>
+      </c>
+      <c r="F272" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G272" t="n">
+        <v>469.2</v>
+      </c>
+      <c r="I272" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>رينفي</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>#1: استيكر ترقيم مقاس 10*10 سم - من1-33 مكررة 6 مرات بالعربي والإنجليزي | Qty: 396 | Price: 3.5 | Total: 1386 | VAT: 207.9; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Quotation#233</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>1386</v>
+      </c>
+      <c r="F273" t="n">
+        <v>207.9</v>
+      </c>
+      <c r="G273" t="n">
+        <v>1593.9</v>
+      </c>
+      <c r="I273" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>نادي بي فيت</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>#1: طباعة شهادة مقاس A4 - مع دعامة (استاند) أكريلك مطبوع | Qty: 16 | Price: 100 | Total: 1600 | VAT: 240; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Quotation#239, Invoice#412, QB#5200</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F274" t="n">
+        <v>240</v>
+      </c>
+      <c r="G274" t="n">
+        <v>1840</v>
+      </c>
+      <c r="I274" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>نادي بي فيت</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>#1: بطاقات مقاس 18*7 سم - تصاميم مختلفة | Qty: 24 | Price: 2.5 | Total: 60 | VAT: 9; #2: توصيل | Qty: 1 | Price: 30 | Total: 30 | VAT: 4.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Quotation#239, Invoice#412, QB#5201</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>90</v>
+      </c>
+      <c r="F275" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G275" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="I275" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>شركة كيري</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>#1: استاند رول أب مقاس 120*200 سم - سيفتي | Qty: 2 | Price: 380 | Total: 760 | VAT: 114; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>760</v>
+      </c>
+      <c r="F276" t="n">
+        <v>114</v>
+      </c>
+      <c r="G276" t="n">
+        <v>874</v>
+      </c>
+      <c r="I276" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>شركة كيري</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>#1: رول أب اليوم الوطني - مقاس 150*200 سم | Qty: 2 | Price: 480 | Total: 960 | VAT: 144; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>960</v>
+      </c>
+      <c r="F277" t="n">
+        <v>144</v>
+      </c>
+      <c r="G277" t="n">
+        <v>1104</v>
+      </c>
+      <c r="I277" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>خبراء قطع المعدات</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>#1: تصميم الافتتاح الكبير | Qty: 1 | Price: 80 | Total: 80 | VAT: 12; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>80</v>
+      </c>
+      <c r="F278" t="n">
+        <v>12</v>
+      </c>
+      <c r="G278" t="n">
+        <v>92</v>
+      </c>
+      <c r="I278" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>مستشفى سليمان فقيه</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>#1: تفصيل دروع صغيرة مقاس 17*25 سم - أكريليك أسود 6ملم - طبقة ثانية أكريليك أبيض مطبوع يو في مع استيكر بالاسماء - قاعدة طبقتين 8 ملم - دولاب قطيفة | Qty: 101 | Price: 196.10 | Total: 19806.1 | VAT: 2970.91; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Quotation#230, Invoice#411</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>19806.1</v>
+      </c>
+      <c r="F279" t="n">
+        <v>2970.91</v>
+      </c>
+      <c r="G279" t="n">
+        <v>22777.01</v>
+      </c>
+      <c r="I279" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>أم عبدالمحسن</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>#1: كتاب تغليف حلزوني 109 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 120 | Total: 120 | VAT: 0; #2: كتاب تغليف حلزوني 22 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 22 | Total: 22 | VAT: 0; #3: كتاب تغليف حلزوني 16 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 16 | Total: 16 | VAT: 0; #4: كتاب تغليف حلزوني 32 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 32 | Total: 32 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>190</v>
+      </c>
+      <c r="F280" t="n">
+        <v>0</v>
+      </c>
+      <c r="G280" t="n">
+        <v>190</v>
+      </c>
+      <c r="I280" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>أم عبدالمحسن</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>#1: كتاب تغليف حلزوني 23 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 30 | Total: 30 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>30</v>
+      </c>
+      <c r="F281" t="n">
+        <v>0</v>
+      </c>
+      <c r="G281" t="n">
+        <v>30</v>
+      </c>
+      <c r="I281" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>مجمع نقاء الطبي</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>#1: بطاقة شروق سويلم البلوي | Qty: 1 | Price: 46 | Total: 46 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>46</v>
+      </c>
+      <c r="F282" t="n">
+        <v>0</v>
+      </c>
+      <c r="G282" t="n">
+        <v>46</v>
+      </c>
+      <c r="I282" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>معهد اللغة الإنجليزية - جامعة الملك عبدالعزيز برابغ</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2025-09-09</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>#1: تصميم إعلان مقاس A3 | Qty: 1 | Price: 60 | Total: 60 | VAT: 9; #2: طباعة إعلان مقاس A3 على استيكر بلاستيك | Qty: 5 | Price: 20 | Total: 100 | VAT: 15; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>160</v>
+      </c>
+      <c r="F283" t="n">
+        <v>24</v>
+      </c>
+      <c r="G283" t="n">
+        <v>184</v>
+      </c>
+      <c r="I283" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>معهد اللغة الإنجليزية - جامعة الملك عبدالعزيز برابغ</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>#1: تصميم لوحة مركز الكتابة | Qty: 1 | Price: 60 | Total: 60 | VAT: 9; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>60</v>
+      </c>
+      <c r="F284" t="n">
+        <v>9</v>
+      </c>
+      <c r="G284" t="n">
+        <v>69</v>
+      </c>
+      <c r="I284" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>معهد اللغة الإنجليزية - جامعة الملك عبدالعزيز برابغ</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>#1: لوحة أكريليك مقاس 40*30 سم - سماكة 6ملم - مع أخرام ومسامير | Qty: 1 | Price: 200 | Total: 200 | VAT: 30; #2: تصميم لوحة خدمات Academic Writing Center | Qty: 1 | Price: 60 | Total: 60 | VAT: 9; #3: تصميم لوحة باركود وحدة الإرشاد | Qty: 1 | Price: 60 | Total: 60 | VAT: 9; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>320</v>
+      </c>
+      <c r="F285" t="n">
+        <v>48</v>
+      </c>
+      <c r="G285" t="n">
+        <v>368</v>
+      </c>
+      <c r="I285" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>دكتورة براء رجب</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>#1: استيكر مقاس 110*15 سم | Qty: 2 | Price: 40.25 | Total: 80.5 | VAT: 0; #2: استيكر مقاس 60*40 سم | Qty: 3 | Price: 46 | Total: 138 | VAT: 0; #3: استيكر مقاس 60*70 سم | Qty: 1 | Price: 57.5 | Total: 57.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>276</v>
+      </c>
+      <c r="F286" t="n">
+        <v>0</v>
+      </c>
+      <c r="G286" t="n">
+        <v>276</v>
+      </c>
+      <c r="I286" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>سعيد الشيخي</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>#1: لوحة مكتبية - أ/سعيد الشيخي | Qty: 1 | Price: 250 | Total: 250 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>250</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0</v>
+      </c>
+      <c r="G287" t="n">
+        <v>250</v>
+      </c>
+      <c r="I287" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>سامية العتيبي</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>#1: فولدرات اليوم الوطني | Qty: 5 | Price: 17.25 | Total: 86.25 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>QB#5204</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>86.25</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0</v>
+      </c>
+      <c r="G288" t="n">
+        <v>86.25</v>
+      </c>
+      <c r="I288" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>سامية العتيبي</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>#1: فولدرات اليوم الوطني لصاحبتها | Qty: 2 | Price: 17.25 | Total: 34.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
+      <c r="G289" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I289" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>رماه</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>#1: بطاقة آي دي إضافية | Qty: 1 | Price: 80.5 | Total: 80.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0</v>
+      </c>
+      <c r="G290" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="I290" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>أسامة الأحمدي</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>#1: رول أب كلية علوم البحار | Qty: 1 | Price: 150 | Total: 150 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>150</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0</v>
+      </c>
+      <c r="G291" t="n">
+        <v>150</v>
+      </c>
+      <c r="I291" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>سارة - شعبيات سعودية</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>#1: استيكر مقاس 9*7 سم - 7 نماذج - من كل نموذج 9 حبات | Qty: 63 | Price: 1.15 | Total: 72.45 | VAT: 0; #2: استيكر مقاس 9*7 سم - بهارات مشكلة | Qty: 37 | Price: 1.15 | Total: 42.55 | VAT: 0; #3: استيكر مقاس 9*12 سم - نموذجين - من كل نموذج 30 حبات | Qty: 60 | Price: 1.38 | Total: 82.8 | VAT: 0; #4: استيكر مقاس 9*12 سم - القهوة السعودية | Qty: 40 | Price: 1.38 | Total: 55.2 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>253</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0</v>
+      </c>
+      <c r="G292" t="n">
+        <v>253</v>
+      </c>
+      <c r="I292" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>مدرسة 176 - أسماء عليثة الحازمي</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>#1: تغيير جلدة ختم | Qty: 1 | Price: 46 | Total: 46 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>46</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0</v>
+      </c>
+      <c r="G293" t="n">
+        <v>46</v>
+      </c>
+      <c r="I293" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>نجود - فلين</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>#1: أغلفة ملفات طباعة ديجيتال | Qty: 5 | Price: 16 | Total: 80 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>80</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0</v>
+      </c>
+      <c r="G294" t="n">
+        <v>80</v>
+      </c>
+      <c r="I294" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>خبراء الفلاتر</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>#1: استيكر أصناف | Qty: 30 | Price: 0.8 | Total: 24 | VAT: 3.6; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>24</v>
+      </c>
+      <c r="F295" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G295" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I295" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>بدور المحمدي</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2025-08-25</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>#1: فلين 50*70 سم | Qty: 1 | Price: 50 | Total: 50 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>QB#5189</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>50</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
+      <c r="G296" t="n">
+        <v>50</v>
+      </c>
+      <c r="I296" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix logging setup: move middleware and exception handler below FastAPI app creation. Add error, access, audit, and IP logging. Fix Reference filter crash in frontend. Update Excel backups. All changes since last commit.
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I296"/>
+  <dimension ref="A1:I311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6648,17 +6648,22 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>#1: لوحة فوركس مقاس A4 - مع قاعدة أكريليك مطبوعة يو في | Qty: 2 | Price: 100 | Total: 200 | VAT: 30; #2: لوحة فوركس مقاس A5 - مع قاعدة أكريليك مطبوعة يو في | Qty: 2 | Price: 70 | Total: 140 | VAT: 21</t>
+          <t>#1: لوحة فوركس مقاس A4 - مع قاعدة أكريليك مطبوعة يو في | Qty: 2 | Price: 100 | Total: 200 | VAT: 30; #2: لوحة فوركس مقاس A5 - مع قاعدة أكريليك مطبوعة يو في | Qty: 2 | Price: 80 | Total: 160 | VAT: 24; #3: لوحة فوركس مقاس 38*10 سم- مع قاعدة أكريليك مطبوعة يو في | Qty: 5 | Price: 60 | Total: 300 | VAT: 45; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Quotation#246</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>340</v>
+        <v>660</v>
       </c>
       <c r="F196" t="n">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="G196" t="n">
-        <v>391</v>
+        <v>759</v>
       </c>
       <c r="I196" t="b">
         <v>0</v>
@@ -7016,7 +7021,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Invoice#392</t>
+          <t>Invoice#392, QB#5210</t>
         </is>
       </c>
       <c r="E208" t="n">
@@ -7029,7 +7034,7 @@
         <v>230</v>
       </c>
       <c r="I208" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -7062,7 +7067,6 @@
       <c r="G209" t="n">
         <v>402.5</v>
       </c>
-      <c r="H209" t="inlineStr"/>
       <c r="I209" t="b">
         <v>1</v>
       </c>
@@ -7083,6 +7087,11 @@
           <t>#1: ختم دائري معتمد - بالعنوان - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; #2: ختم دائري معتمد - فرع الطائف - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>QB#5208</t>
+        </is>
+      </c>
       <c r="E210" t="n">
         <v>276</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>276</v>
       </c>
       <c r="I210" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211">
@@ -7177,7 +7186,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Invoice#396</t>
+          <t>Invoice#396, QB#5212</t>
         </is>
       </c>
       <c r="E213" t="n">
@@ -7190,7 +7199,7 @@
         <v>92</v>
       </c>
       <c r="I213" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -7209,6 +7218,11 @@
           <t>#1: كروت بزنس - كوشيه سلوفان مطفي وجهين | Qty: 200 | Price: 0.517 | Total: 103.4 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>QB#5214</t>
+        </is>
+      </c>
       <c r="E214" t="n">
         <v>103.4</v>
       </c>
@@ -7219,7 +7233,7 @@
         <v>103.4</v>
       </c>
       <c r="I214" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215">
@@ -7267,6 +7281,11 @@
           <t>#1: كرت بزنس - كوشيه مطفي وجهين | Qty: 50 | Price: 1.38 | Total: 69 | VAT: 0; #2: كرت شكر - 15*10 سم | Qty: 50 | Price: 2.76 | Total: 138 | VAT: 0; #3: سليف علبة مقاس 10*80 سم | Qty: 30 | Price: 10 | Total: 300 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>QB#5213</t>
+        </is>
+      </c>
       <c r="E216" t="n">
         <v>507</v>
       </c>
@@ -7277,7 +7296,7 @@
         <v>507</v>
       </c>
       <c r="I216" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -7325,6 +7344,11 @@
           <t>#1: ختم مؤسسة دائري - R538 | Qty: 1 | Price: 138 | Total: 138 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>QB#5215</t>
+        </is>
+      </c>
       <c r="E218" t="n">
         <v>138</v>
       </c>
@@ -7335,7 +7359,7 @@
         <v>138</v>
       </c>
       <c r="I218" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -7448,7 +7472,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Invoice#405</t>
+          <t>Invoice#405, QB#5218</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -7461,7 +7485,7 @@
         <v>30</v>
       </c>
       <c r="I222" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223">
@@ -7509,6 +7533,11 @@
           <t>#1: ختم الدكتورة شروق عابد - S852 | Qty: 1 | Price: 80 | Total: 80 | VAT: 0; #2: ختم الدكتورة شروق عابد - S854 | Qty: 1 | Price: 120 | Total: 120 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>QB#5219</t>
+        </is>
+      </c>
       <c r="E224" t="n">
         <v>200</v>
       </c>
@@ -7518,8 +7547,9 @@
       <c r="G224" t="n">
         <v>200</v>
       </c>
+      <c r="H224" t="inlineStr"/>
       <c r="I224" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225">
@@ -7777,7 +7807,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Quotation#220</t>
+          <t>Quotation#220, QB#5209</t>
         </is>
       </c>
       <c r="E233" t="n">
@@ -9273,6 +9303,11 @@
           <t>#1: كتاب تغليف حلزوني 109 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 120 | Total: 120 | VAT: 0; #2: كتاب تغليف حلزوني 22 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 22 | Total: 22 | VAT: 0; #3: كتاب تغليف حلزوني 16 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 16 | Total: 16 | VAT: 0; #4: كتاب تغليف حلزوني 32 صفحة داخلية - وودفري 100 جرام | Qty: 1 | Price: 32 | Total: 32 | VAT: 0; Discount: 0</t>
         </is>
       </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>QB#5217</t>
+        </is>
+      </c>
       <c r="E280" t="n">
         <v>190</v>
       </c>
@@ -9283,7 +9318,7 @@
         <v>190</v>
       </c>
       <c r="I280" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="281">
@@ -9758,6 +9793,476 @@
       </c>
       <c r="I296" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>محمد صولان</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2025-09-16</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>#1: استيكر مقاس 60*118 سم - مسلفن مطفي | Qty: 3 | Price: 46 | Total: 138 | VAT: 0; #2: استيكر مقاس 27*52 سم - مسلفن مطفي | Qty: 2 | Price: 17.25 | Total: 34.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0</v>
+      </c>
+      <c r="G297" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="I297" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>مصنع عاشق العود</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>#1: كروت عمل مقاس 9*5 سم - 10 نماذج (200 من كل نموذج) | Qty: 10 | Price: 92 | Total: 920 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>920</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0</v>
+      </c>
+      <c r="G298" t="n">
+        <v>920</v>
+      </c>
+      <c r="I298" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>شركة نخبة الصلابة - عمرو كتبي</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>#1: تصميم شعار | Qty: 1 | Price: 345 | Total: 345 | VAT: 0; #2: طباعة ورق خطابات فاخر | Qty: 100 | Price: 1.725 | Total: 172.5 | VAT: 0; #3: ختم دائري R538 | Qty: 2 | Price: 138 | Total: 276 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>793.5</v>
+      </c>
+      <c r="F299" t="n">
+        <v>0</v>
+      </c>
+      <c r="G299" t="n">
+        <v>793.5</v>
+      </c>
+      <c r="I299" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>قرطاسية المودة</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>#1: استيكر ملف | Qty: 2 | Price: 15 | Total: 30 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>30</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0</v>
+      </c>
+      <c r="G300" t="n">
+        <v>30</v>
+      </c>
+      <c r="I300" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>نادي الاتحاد</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>#1: فوركس إعلان بدون قاعدية مقاس A4 | Qty: 3 | Price: 80 | Total: 240 | VAT: 36; #2: فوركس إعلان بدون قاعدية مقاس A5 | Qty: 3 | Price: 60 | Total: 180 | VAT: 27; #3: فوركس إعلان بدون قاعدية مقاس 38*10 | Qty: 3 | Price: 50 | Total: 150 | VAT: 22.5; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Quotation#247</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>570</v>
+      </c>
+      <c r="F301" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="G301" t="n">
+        <v>655.5</v>
+      </c>
+      <c r="I301" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>بن حمران</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>#1: كتاب الواجبات والأسس الشرعية - دليل المتدرب | Qty: 230 | Price: 32.5 | Total: 7475 | VAT: 1121.25; #2: كتاب مراحل النمو - دليل المتدرب | Qty: 230 | Price: 34.1 | Total: 7843 | VAT: 1176.45; #3: كتاب غرس القيم وتعديل السلوك | Qty: 230 | Price: 34.5 | Total: 7935 | VAT: 1190.25; #4: كراسة المشارك للبرنامج التدريبي | Qty: 230 | Price: 11.2 | Total: 2576 | VAT: 386.4; #5: دليل ممارسات مبادرة ألفة | Qty: 230 | Price: 10.4 | Total: 2392 | VAT: 358.8; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Quotation#223, Invoice#393, QB#5211</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>28221</v>
+      </c>
+      <c r="F302" t="n">
+        <v>4233.15</v>
+      </c>
+      <c r="G302" t="n">
+        <v>32454.15</v>
+      </c>
+      <c r="I302" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>نادي بي فيت</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2025-09-22</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>#1: طباعة عقد على ورق مقاس A4 - وودفري - 100 جرام وجه واحد | Qty: 100 | Price: 0.8 | Total: 80 | VAT: 12; #2: كروت مقاس 18*8 سم - طباعة وجه واحد | Qty: 30 | Price: 2 | Total: 60 | VAT: 9; #3: بوست - ورق 300 جرام مقاس A4 مطبوع وجه واحد | Qty: 4 | Price: 10 | Total: 40 | VAT: 6; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Invoice#414</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>180</v>
+      </c>
+      <c r="F303" t="n">
+        <v>27</v>
+      </c>
+      <c r="G303" t="n">
+        <v>207</v>
+      </c>
+      <c r="I303" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>مركز منارات الطفولة - مارية القبطية</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2025-08-17</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>#1: سند صرف - 1+2 - لون أزرق - 0001 | Qty: 10 | Price: 23 | Total: 230 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>QB#5173</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>230</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0</v>
+      </c>
+      <c r="G304" t="n">
+        <v>230</v>
+      </c>
+      <c r="I304" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>ريم الشهري - الشؤون الصحية بالحرس الوطني</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>#1: فلاير مقاس A4 - 6 نماذج- من كل نموذج 20 | Qty: 120 | Price: 2.07 | Total: 248.4 | VAT: 0; #2: بطاقة مقاس 10.5*7.5 سم - 5نماذج - 15 من كل نموذج | Qty: 75 | Price: 1.15 | Total: 86.25 | VAT: 0; Discount: 1.15</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Quotation#252</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="n">
+        <v>333.5</v>
+      </c>
+      <c r="I305" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>أم عبدالله - كروت اليوم الوطني</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>#1: كرت مقاس 9*10 سم - وجه واحد بدون سلوفان | Qty: 1000 | Price: 0.23 | Total: 230 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>230</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="n">
+        <v>230</v>
+      </c>
+      <c r="I306" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>منال الشريف</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>#1: فلين كامل | Qty: 1 | Price: 80.5 | Total: 80.5 | VAT: 0; #2: كرت مقاس A6 - وجه واحد - نموذجين - 8 من كل واحد | Qty: 16 | Price: 2.875 | Total: 46 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="I307" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>الرعاية المنزلية - جامعة الملك عبدالعزيز</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>#1: طباعة وتغيير رول أب مقاس 85*200 سم | Qty: 2 | Price: 100 | Total: 200 | VAT: 30; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Invoice#417</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>200</v>
+      </c>
+      <c r="F308" t="n">
+        <v>30</v>
+      </c>
+      <c r="G308" t="n">
+        <v>230</v>
+      </c>
+      <c r="I308" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>دوت وان كافيه</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2025-09-24</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>#1: تغيير رول أب قري باك 85*200 سم | Qty: 3 | Price: 138 | Total: 414 | VAT: 0; #2: بروشور مقاس A5 وجه واحد | Qty: 100 | Price: 1.725 | Total: 172.5 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>586.5</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" t="n">
+        <v>586.5</v>
+      </c>
+      <c r="I309" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>ذا أوفيس TheOffice</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2025-09-22</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>#1: ورق مقوى مقاس A4 - 6 نماذج - وجهين | Qty: 12 | Price: 5 | Total: 60 | VAT: 9; #2: دانقلر مربع مقاس 30*30 سم - مطبوع وجهين | Qty: 12 | Price: 13.35 | Total: 160.2 | VAT: 24.03; Discount: 0</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Invoice#415</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>220.2</v>
+      </c>
+      <c r="F310" t="n">
+        <v>33.03</v>
+      </c>
+      <c r="G310" t="n">
+        <v>253.23</v>
+      </c>
+      <c r="I310" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>خالد أبو سعيد</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2025-08-19</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>#1: بوكس مع سليف مقاس 19*10 *7 سم - نموذجين | Qty: 500 | Price: 4.5 | Total: 2250 | VAT: 0; #2: استيكرات طقوس | Qty: 200 | Price: 0.3 | Total: 60 | VAT: 0; Discount: 0</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>2310</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
+        <v>2310</v>
+      </c>
+      <c r="I311" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>